<commit_message>
feat: improve batch inversion data workflow
- parameterize monitor extraction and batch input selection
- deduplicate SHSH station sheets and refresh monitoring workbooks
- initialize sources from raw observation peaks and relax Q bounds
</commit_message>
<xml_diff>
--- a/data/shsh_js/concentration.xlsx
+++ b/data/shsh_js/concentration.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,22 +453,22 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>二工区东北园区站(亚南)</t>
+          <t>碳谷绿湾南部园区站（抚佳）</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>二工区南部园区站（抚佳）</t>
+          <t>碳谷绿湾东北园区站 (亚南)</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>二工区边界新联站</t>
+          <t>碳谷绿湾边界新联站</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>二工区边界国贸站</t>
+          <t>碳谷绿湾边界国贸站</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
@@ -484,521 +484,533 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46121.29166666666</v>
+        <v>46186</v>
       </c>
       <c r="B2" t="n">
-        <v>7.6</v>
+        <v>26</v>
       </c>
       <c r="C2" t="n">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>2.91</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>6.4</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>3.9</v>
+        <v>19.05</v>
       </c>
       <c r="H2" t="n">
-        <v>1.5</v>
+        <v>2.11</v>
       </c>
       <c r="I2" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1.8</v>
-      </c>
+        <v>5.57</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>3.9</v>
+        <v>0.9</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46121.33333333334</v>
+        <v>46186.04166666666</v>
       </c>
       <c r="B3" t="n">
-        <v>7.7</v>
+        <v>59.86</v>
       </c>
       <c r="C3" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>6.9</v>
+        <v>2.12</v>
       </c>
       <c r="E3" t="n">
-        <v>3.7</v>
+        <v>0.24</v>
       </c>
       <c r="F3" t="n">
-        <v>6.8</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>3.8</v>
+        <v>11.15</v>
       </c>
       <c r="H3" t="n">
-        <v>1.5</v>
+        <v>1.48</v>
       </c>
       <c r="I3" t="n">
-        <v>9</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1.9</v>
-      </c>
+        <v>4.89</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
-        <v>4</v>
+        <v>0.78</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46121.375</v>
+        <v>46186.08333333334</v>
       </c>
       <c r="B4" t="n">
-        <v>7.9</v>
+        <v>208.94</v>
       </c>
       <c r="C4" t="n">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>6.5</v>
+        <v>1.66</v>
       </c>
       <c r="E4" t="n">
-        <v>2.6</v>
+        <v>0.32</v>
       </c>
       <c r="F4" t="n">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>5.3</v>
+        <v>2.86</v>
       </c>
       <c r="H4" t="n">
-        <v>3.4</v>
+        <v>1.93</v>
       </c>
       <c r="I4" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="J4" t="n">
-        <v>2.9</v>
-      </c>
+        <v>3.32</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
-        <v>4.3</v>
+        <v>0.6</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46121.41666666666</v>
+        <v>46186.125</v>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>159.72</v>
       </c>
       <c r="C5" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>6.8</v>
+        <v>2.11</v>
       </c>
       <c r="E5" t="n">
-        <v>12.5</v>
+        <v>0.48</v>
       </c>
       <c r="F5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>5.2</v>
+        <v>13.61</v>
       </c>
       <c r="H5" t="n">
-        <v>2.9</v>
+        <v>1.07</v>
       </c>
       <c r="I5" t="n">
-        <v>7</v>
-      </c>
-      <c r="J5" t="n">
-        <v>4.1</v>
-      </c>
+        <v>2.78</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
-        <v>7.4</v>
+        <v>0.57</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46121.45833333334</v>
+        <v>46186.16666666666</v>
       </c>
       <c r="B6" t="n">
-        <v>8.699999999999999</v>
+        <v>285.62</v>
       </c>
       <c r="C6" t="n">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>7.7</v>
+        <v>1.81</v>
       </c>
       <c r="E6" t="n">
-        <v>12.6</v>
+        <v>0.06</v>
       </c>
       <c r="F6" t="n">
-        <v>7.7</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>4.7</v>
+        <v>0.74</v>
       </c>
       <c r="H6" t="n">
-        <v>2.8</v>
+        <v>0.97</v>
       </c>
       <c r="I6" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="J6" t="n">
-        <v>4.1</v>
-      </c>
+        <v>2.12</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
-        <v>5.7</v>
+        <v>0.59</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46121.5</v>
+        <v>46186.20833333334</v>
       </c>
       <c r="B7" t="n">
-        <v>8.5</v>
+        <v>84.68000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>6.2</v>
+        <v>1.77</v>
       </c>
       <c r="E7" t="n">
-        <v>4.5</v>
+        <v>0.88</v>
       </c>
       <c r="F7" t="n">
-        <v>6.6</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>3.9</v>
+        <v>0.84</v>
       </c>
       <c r="H7" t="n">
-        <v>2.5</v>
+        <v>0.78</v>
       </c>
       <c r="I7" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="J7" t="n">
-        <v>2.3</v>
-      </c>
+        <v>2.01</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
-        <v>4.4</v>
+        <v>0.7</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46121.54166666666</v>
+        <v>46186.25</v>
       </c>
       <c r="B8" t="n">
-        <v>8.1</v>
+        <v>382.92</v>
       </c>
       <c r="C8" t="n">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>243.4</v>
+        <v>1.98</v>
       </c>
       <c r="E8" t="n">
-        <v>18.9</v>
+        <v>0.05</v>
       </c>
       <c r="F8" t="n">
-        <v>7.1</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>2.8</v>
+        <v>0.96</v>
       </c>
       <c r="I8" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="J8" t="n">
-        <v>3.5</v>
-      </c>
+        <v>1.57</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>5.5</v>
+        <v>0.74</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46121.58333333334</v>
+        <v>46186.29166666666</v>
       </c>
       <c r="B9" t="n">
-        <v>8.9</v>
+        <v>237.6</v>
       </c>
       <c r="C9" t="n">
-        <v>4.5</v>
+        <v>0.88</v>
       </c>
       <c r="D9" t="n">
-        <v>14.9</v>
+        <v>2.67</v>
       </c>
       <c r="E9" t="n">
-        <v>10.7</v>
+        <v>16.02</v>
       </c>
       <c r="F9" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>4.5</v>
+        <v>0.96</v>
       </c>
       <c r="H9" t="n">
-        <v>2.6</v>
+        <v>0.92</v>
       </c>
       <c r="I9" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="J9" t="n">
-        <v>3.4</v>
-      </c>
+        <v>0.95</v>
+      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>6.3</v>
+        <v>0.71</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46121.625</v>
+        <v>46186.33333333334</v>
       </c>
       <c r="B10" t="n">
-        <v>10.9</v>
+        <v>154.3</v>
       </c>
       <c r="C10" t="n">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>11.6</v>
+        <v>4.18</v>
       </c>
       <c r="E10" t="n">
-        <v>18.4</v>
+        <v>2.76</v>
       </c>
       <c r="F10" t="n">
-        <v>8.300000000000001</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>5.8</v>
+        <v>2.04</v>
       </c>
       <c r="H10" t="n">
-        <v>3.3</v>
+        <v>0.48</v>
       </c>
       <c r="I10" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="J10" t="n">
-        <v>4.5</v>
-      </c>
+        <v>1.6</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>7.2</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46121.66666666666</v>
+        <v>46186.375</v>
       </c>
       <c r="B11" t="n">
-        <v>89.7</v>
+        <v>29.75</v>
       </c>
       <c r="C11" t="n">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>8.6</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>11.3</v>
+        <v>0.35</v>
       </c>
       <c r="F11" t="n">
-        <v>7.7</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>5.6</v>
+        <v>1.06</v>
       </c>
       <c r="H11" t="n">
-        <v>2.8</v>
+        <v>0.66</v>
       </c>
       <c r="I11" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="J11" t="n">
-        <v>3.8</v>
-      </c>
+        <v>1.54</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>7.3</v>
+        <v>0.79</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46121.70833333334</v>
+        <v>46186.41666666666</v>
       </c>
       <c r="B12" t="n">
-        <v>133.3</v>
+        <v>1.52</v>
       </c>
       <c r="C12" t="n">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>8.9</v>
+        <v>2.49</v>
       </c>
       <c r="E12" t="n">
-        <v>6.1</v>
+        <v>0.41</v>
       </c>
       <c r="F12" t="n">
-        <v>8.199999999999999</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>5.3</v>
+        <v>13.14</v>
       </c>
       <c r="H12" t="n">
-        <v>3.4</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="J12" t="n">
-        <v>4.2</v>
-      </c>
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>6.8</v>
+        <v>0.52</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46121.75</v>
+        <v>46186.45833333334</v>
       </c>
       <c r="B13" t="n">
-        <v>7.4</v>
+        <v>3.62</v>
       </c>
       <c r="C13" t="n">
-        <v>3.7</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>9.6</v>
+        <v>2.64</v>
       </c>
       <c r="E13" t="n">
-        <v>6.2</v>
+        <v>0.62</v>
       </c>
       <c r="F13" t="n">
-        <v>8.1</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>4.8</v>
+        <v>9.98</v>
       </c>
       <c r="H13" t="n">
-        <v>2.7</v>
+        <v>6.56</v>
       </c>
       <c r="I13" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="J13" t="n">
-        <v>3.2</v>
-      </c>
+        <v>1.35</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>4.8</v>
+        <v>0.61</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46121.79166666666</v>
+        <v>46186.5</v>
       </c>
       <c r="B14" t="n">
-        <v>5.6</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
-        <v>3.7</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>9.699999999999999</v>
+        <v>8.34</v>
       </c>
       <c r="E14" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>8.6</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>5.6</v>
+        <v>15.38</v>
       </c>
       <c r="H14" t="n">
-        <v>3.7</v>
+        <v>2.5</v>
       </c>
       <c r="I14" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="J14" t="n">
-        <v>4</v>
-      </c>
+        <v>1.09</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="n">
-        <v>8.1</v>
+        <v>0.55</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>硫化氢(H₂S)</t>
+          <t>乙烯</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46186.54166666666</v>
+      </c>
+      <c r="B15" t="n">
+        <v>151.35</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>乙烯</t>
         </is>
       </c>
     </row>

</xml_diff>